<commit_message>
docs: standardize table captions
</commit_message>
<xml_diff>
--- a/docs/assets/protocol/cavo-realtek-watch-protocol.xlsx
+++ b/docs/assets/protocol/cavo-realtek-watch-protocol.xlsx
@@ -9514,7 +9514,7 @@
     <t xml:space="preserve">例如 00 01 表示今天和昨天</t>
   </si>
   <si>
-    <t xml:space="preserve">类型和 index 取交集：</t>
+    <t xml:space="preserve">表：筛选结果示例</t>
   </si>
   <si>
     <t xml:space="preserve">想要</t>
@@ -12255,6 +12255,15 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">表：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
         <rFont val="宋体"/>
         <family val="2"/>
         <charset val="1"/>
@@ -12268,7 +12277,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">的设置（</t>
+      <t xml:space="preserve">设置（</t>
     </r>
     <r>
       <rPr>
@@ -12287,26 +12296,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">，和设置命令里自动监测的格式一样，</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="宋体"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">SDK </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">可以共用编解码）：</t>
+      <t xml:space="preserve">，格式同自动监测）</t>
     </r>
   </si>
   <si>
@@ -12480,6 +12470,15 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">表：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
         <rFont val="宋体"/>
         <family val="2"/>
         <charset val="1"/>
@@ -12531,7 +12530,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">）：</t>
+      <t xml:space="preserve">）</t>
     </r>
   </si>
   <si>
@@ -26842,7 +26841,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="38">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -26972,6 +26971,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="17" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -30818,957 +30821,957 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="35" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="34" t="s">
+      <c r="B1" s="35" t="s">
         <v>91</v>
       </c>
-      <c r="C1" s="34" t="s">
+      <c r="C1" s="35" t="s">
         <v>1497</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="35" t="s">
+      <c r="A2" s="36" t="s">
         <v>1561</v>
       </c>
-      <c r="B2" s="36" t="s">
+      <c r="B2" s="37" t="s">
         <v>1497</v>
       </c>
-      <c r="C2" s="35" t="s">
+      <c r="C2" s="36" t="s">
         <v>1562</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="35" t="s">
+      <c r="A3" s="36" t="s">
         <v>1563</v>
       </c>
-      <c r="B3" s="36" t="s">
+      <c r="B3" s="37" t="s">
         <v>1564</v>
       </c>
-      <c r="C3" s="35" t="s">
+      <c r="C3" s="36" t="s">
         <v>1565</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="35" t="s">
+      <c r="A4" s="36" t="s">
         <v>1566</v>
       </c>
-      <c r="B4" s="36" t="s">
+      <c r="B4" s="37" t="s">
         <v>1567</v>
       </c>
-      <c r="C4" s="35" t="s">
+      <c r="C4" s="36" t="s">
         <v>1568</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="35" t="s">
+      <c r="A5" s="36" t="s">
         <v>1569</v>
       </c>
-      <c r="B5" s="36" t="s">
+      <c r="B5" s="37" t="s">
         <v>1570</v>
       </c>
-      <c r="C5" s="35"/>
+      <c r="C5" s="36"/>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="35" t="s">
+      <c r="A6" s="36" t="s">
         <v>1571</v>
       </c>
-      <c r="B6" s="36" t="s">
+      <c r="B6" s="37" t="s">
         <v>1572</v>
       </c>
-      <c r="C6" s="35"/>
+      <c r="C6" s="36"/>
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="35" t="s">
+      <c r="A7" s="36" t="s">
         <v>1573</v>
       </c>
-      <c r="B7" s="36" t="s">
+      <c r="B7" s="37" t="s">
         <v>1574</v>
       </c>
-      <c r="C7" s="35"/>
+      <c r="C7" s="36"/>
     </row>
     <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="35" t="s">
+      <c r="A8" s="36" t="s">
         <v>1575</v>
       </c>
-      <c r="B8" s="36" t="s">
+      <c r="B8" s="37" t="s">
         <v>1576</v>
       </c>
-      <c r="C8" s="35"/>
+      <c r="C8" s="36"/>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="35" t="s">
+      <c r="A9" s="36" t="s">
         <v>1577</v>
       </c>
-      <c r="B9" s="36" t="s">
+      <c r="B9" s="37" t="s">
         <v>1578</v>
       </c>
-      <c r="C9" s="35"/>
+      <c r="C9" s="36"/>
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="35" t="s">
+      <c r="A10" s="36" t="s">
         <v>1579</v>
       </c>
-      <c r="B10" s="36" t="s">
+      <c r="B10" s="37" t="s">
         <v>1580</v>
       </c>
-      <c r="C10" s="35"/>
+      <c r="C10" s="36"/>
     </row>
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="35" t="s">
+      <c r="A11" s="36" t="s">
         <v>1581</v>
       </c>
-      <c r="B11" s="36" t="s">
+      <c r="B11" s="37" t="s">
         <v>1582</v>
       </c>
-      <c r="C11" s="35"/>
+      <c r="C11" s="36"/>
     </row>
     <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="35" t="s">
+      <c r="A12" s="36" t="s">
         <v>1583</v>
       </c>
-      <c r="B12" s="36" t="s">
+      <c r="B12" s="37" t="s">
         <v>1584</v>
       </c>
-      <c r="C12" s="35"/>
+      <c r="C12" s="36"/>
     </row>
     <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="35" t="s">
+      <c r="A13" s="36" t="s">
         <v>1585</v>
       </c>
-      <c r="B13" s="36" t="s">
+      <c r="B13" s="37" t="s">
         <v>1586</v>
       </c>
-      <c r="C13" s="35"/>
+      <c r="C13" s="36"/>
     </row>
     <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="35" t="s">
+      <c r="A14" s="36" t="s">
         <v>1587</v>
       </c>
-      <c r="B14" s="36" t="s">
+      <c r="B14" s="37" t="s">
         <v>1588</v>
       </c>
-      <c r="C14" s="35"/>
+      <c r="C14" s="36"/>
     </row>
     <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="35" t="s">
+      <c r="A15" s="36" t="s">
         <v>1589</v>
       </c>
-      <c r="B15" s="36" t="s">
+      <c r="B15" s="37" t="s">
         <v>1590</v>
       </c>
-      <c r="C15" s="35"/>
+      <c r="C15" s="36"/>
     </row>
     <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="35" t="s">
+      <c r="A16" s="36" t="s">
         <v>1591</v>
       </c>
-      <c r="B16" s="36" t="s">
+      <c r="B16" s="37" t="s">
         <v>1592</v>
       </c>
-      <c r="C16" s="35"/>
+      <c r="C16" s="36"/>
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="35" t="s">
+      <c r="A17" s="36" t="s">
         <v>1593</v>
       </c>
-      <c r="B17" s="36" t="s">
+      <c r="B17" s="37" t="s">
         <v>1594</v>
       </c>
-      <c r="C17" s="35"/>
+      <c r="C17" s="36"/>
     </row>
     <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="35" t="s">
+      <c r="A18" s="36" t="s">
         <v>1595</v>
       </c>
-      <c r="B18" s="36" t="s">
+      <c r="B18" s="37" t="s">
         <v>1596</v>
       </c>
-      <c r="C18" s="35"/>
+      <c r="C18" s="36"/>
     </row>
     <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="35" t="s">
+      <c r="A19" s="36" t="s">
         <v>1597</v>
       </c>
-      <c r="B19" s="36" t="s">
+      <c r="B19" s="37" t="s">
         <v>1598</v>
       </c>
-      <c r="C19" s="35"/>
+      <c r="C19" s="36"/>
     </row>
     <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="35" t="s">
+      <c r="A20" s="36" t="s">
         <v>1599</v>
       </c>
-      <c r="B20" s="36" t="s">
+      <c r="B20" s="37" t="s">
         <v>1600</v>
       </c>
-      <c r="C20" s="35"/>
+      <c r="C20" s="36"/>
     </row>
     <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="35" t="s">
+      <c r="A21" s="36" t="s">
         <v>1601</v>
       </c>
-      <c r="B21" s="36" t="s">
+      <c r="B21" s="37" t="s">
         <v>1602</v>
       </c>
-      <c r="C21" s="35"/>
+      <c r="C21" s="36"/>
     </row>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="35" t="s">
+      <c r="A22" s="36" t="s">
         <v>1603</v>
       </c>
-      <c r="B22" s="36" t="s">
+      <c r="B22" s="37" t="s">
         <v>1604</v>
       </c>
-      <c r="C22" s="35"/>
+      <c r="C22" s="36"/>
     </row>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="35" t="s">
+      <c r="A23" s="36" t="s">
         <v>1605</v>
       </c>
-      <c r="B23" s="36" t="s">
+      <c r="B23" s="37" t="s">
         <v>1606</v>
       </c>
-      <c r="C23" s="35"/>
+      <c r="C23" s="36"/>
     </row>
     <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="35" t="s">
+      <c r="A24" s="36" t="s">
         <v>1607</v>
       </c>
-      <c r="B24" s="36" t="s">
+      <c r="B24" s="37" t="s">
         <v>1608</v>
       </c>
-      <c r="C24" s="35"/>
+      <c r="C24" s="36"/>
     </row>
     <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="35" t="s">
+      <c r="A25" s="36" t="s">
         <v>1609</v>
       </c>
-      <c r="B25" s="36" t="s">
+      <c r="B25" s="37" t="s">
         <v>1610</v>
       </c>
-      <c r="C25" s="35"/>
+      <c r="C25" s="36"/>
     </row>
     <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="35" t="s">
+      <c r="A26" s="36" t="s">
         <v>1611</v>
       </c>
-      <c r="B26" s="36" t="s">
+      <c r="B26" s="37" t="s">
         <v>1612</v>
       </c>
-      <c r="C26" s="35"/>
+      <c r="C26" s="36"/>
     </row>
     <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="35" t="s">
+      <c r="A27" s="36" t="s">
         <v>1613</v>
       </c>
-      <c r="B27" s="36" t="s">
+      <c r="B27" s="37" t="s">
         <v>1614</v>
       </c>
-      <c r="C27" s="35"/>
+      <c r="C27" s="36"/>
     </row>
     <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="35" t="s">
+      <c r="A28" s="36" t="s">
         <v>1615</v>
       </c>
-      <c r="B28" s="36" t="s">
+      <c r="B28" s="37" t="s">
         <v>1616</v>
       </c>
-      <c r="C28" s="35"/>
+      <c r="C28" s="36"/>
     </row>
     <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="35" t="s">
+      <c r="A29" s="36" t="s">
         <v>1617</v>
       </c>
-      <c r="B29" s="36" t="s">
+      <c r="B29" s="37" t="s">
         <v>1618</v>
       </c>
-      <c r="C29" s="35"/>
+      <c r="C29" s="36"/>
     </row>
     <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="35" t="s">
+      <c r="A30" s="36" t="s">
         <v>1619</v>
       </c>
-      <c r="B30" s="36" t="s">
+      <c r="B30" s="37" t="s">
         <v>1620</v>
       </c>
-      <c r="C30" s="35"/>
+      <c r="C30" s="36"/>
     </row>
     <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="35" t="s">
+      <c r="A31" s="36" t="s">
         <v>1621</v>
       </c>
-      <c r="B31" s="36" t="s">
+      <c r="B31" s="37" t="s">
         <v>1622</v>
       </c>
-      <c r="C31" s="35"/>
+      <c r="C31" s="36"/>
     </row>
     <row r="32" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="35" t="s">
+      <c r="A32" s="36" t="s">
         <v>1623</v>
       </c>
-      <c r="B32" s="36" t="s">
+      <c r="B32" s="37" t="s">
         <v>1624</v>
       </c>
-      <c r="C32" s="35"/>
+      <c r="C32" s="36"/>
     </row>
     <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="35" t="s">
+      <c r="A33" s="36" t="s">
         <v>1625</v>
       </c>
-      <c r="B33" s="36" t="s">
+      <c r="B33" s="37" t="s">
         <v>1626</v>
       </c>
-      <c r="C33" s="35"/>
+      <c r="C33" s="36"/>
     </row>
     <row r="34" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="35" t="s">
+      <c r="A34" s="36" t="s">
         <v>1627</v>
       </c>
-      <c r="B34" s="36" t="s">
+      <c r="B34" s="37" t="s">
         <v>1628</v>
       </c>
-      <c r="C34" s="35"/>
+      <c r="C34" s="36"/>
     </row>
     <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="35" t="s">
+      <c r="A35" s="36" t="s">
         <v>1629</v>
       </c>
-      <c r="B35" s="36" t="s">
+      <c r="B35" s="37" t="s">
         <v>1630</v>
       </c>
-      <c r="C35" s="35"/>
+      <c r="C35" s="36"/>
     </row>
     <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="35" t="s">
+      <c r="A36" s="36" t="s">
         <v>1631</v>
       </c>
-      <c r="B36" s="36" t="s">
+      <c r="B36" s="37" t="s">
         <v>1632</v>
       </c>
-      <c r="C36" s="35"/>
+      <c r="C36" s="36"/>
     </row>
     <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="35" t="s">
+      <c r="A37" s="36" t="s">
         <v>1633</v>
       </c>
-      <c r="B37" s="36" t="s">
+      <c r="B37" s="37" t="s">
         <v>1634</v>
       </c>
-      <c r="C37" s="35"/>
+      <c r="C37" s="36"/>
     </row>
     <row r="38" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="35" t="s">
+      <c r="A38" s="36" t="s">
         <v>1635</v>
       </c>
-      <c r="B38" s="36" t="s">
+      <c r="B38" s="37" t="s">
         <v>1636</v>
       </c>
-      <c r="C38" s="35"/>
+      <c r="C38" s="36"/>
     </row>
     <row r="39" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="35" t="s">
+      <c r="A39" s="36" t="s">
         <v>1637</v>
       </c>
-      <c r="B39" s="36" t="s">
+      <c r="B39" s="37" t="s">
         <v>1638</v>
       </c>
-      <c r="C39" s="35"/>
+      <c r="C39" s="36"/>
     </row>
     <row r="40" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="35" t="s">
+      <c r="A40" s="36" t="s">
         <v>1639</v>
       </c>
-      <c r="B40" s="36" t="s">
+      <c r="B40" s="37" t="s">
         <v>1640</v>
       </c>
-      <c r="C40" s="35"/>
+      <c r="C40" s="36"/>
     </row>
     <row r="41" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="35" t="s">
+      <c r="A41" s="36" t="s">
         <v>1641</v>
       </c>
-      <c r="B41" s="36" t="s">
+      <c r="B41" s="37" t="s">
         <v>1642</v>
       </c>
-      <c r="C41" s="35"/>
+      <c r="C41" s="36"/>
     </row>
     <row r="42" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="35" t="s">
+      <c r="A42" s="36" t="s">
         <v>1643</v>
       </c>
-      <c r="B42" s="36" t="s">
+      <c r="B42" s="37" t="s">
         <v>1644</v>
       </c>
-      <c r="C42" s="35"/>
+      <c r="C42" s="36"/>
     </row>
     <row r="43" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="35" t="s">
+      <c r="A43" s="36" t="s">
         <v>1645</v>
       </c>
-      <c r="B43" s="36" t="s">
+      <c r="B43" s="37" t="s">
         <v>1646</v>
       </c>
-      <c r="C43" s="35"/>
+      <c r="C43" s="36"/>
     </row>
     <row r="44" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="35" t="s">
+      <c r="A44" s="36" t="s">
         <v>1647</v>
       </c>
-      <c r="B44" s="36" t="s">
+      <c r="B44" s="37" t="s">
         <v>1648</v>
       </c>
-      <c r="C44" s="35"/>
+      <c r="C44" s="36"/>
     </row>
     <row r="45" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="35" t="s">
+      <c r="A45" s="36" t="s">
         <v>1649</v>
       </c>
-      <c r="B45" s="36" t="s">
+      <c r="B45" s="37" t="s">
         <v>1650</v>
       </c>
-      <c r="C45" s="35"/>
+      <c r="C45" s="36"/>
     </row>
     <row r="46" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="35" t="s">
+      <c r="A46" s="36" t="s">
         <v>1651</v>
       </c>
-      <c r="B46" s="36" t="s">
+      <c r="B46" s="37" t="s">
         <v>1652</v>
       </c>
-      <c r="C46" s="35"/>
+      <c r="C46" s="36"/>
     </row>
     <row r="47" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="35" t="s">
+      <c r="A47" s="36" t="s">
         <v>1653</v>
       </c>
-      <c r="B47" s="36" t="s">
+      <c r="B47" s="37" t="s">
         <v>1654</v>
       </c>
-      <c r="C47" s="35"/>
+      <c r="C47" s="36"/>
     </row>
     <row r="48" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="35" t="s">
+      <c r="A48" s="36" t="s">
         <v>1655</v>
       </c>
-      <c r="B48" s="36" t="s">
+      <c r="B48" s="37" t="s">
         <v>1656</v>
       </c>
-      <c r="C48" s="35"/>
+      <c r="C48" s="36"/>
     </row>
     <row r="49" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="35" t="s">
+      <c r="A49" s="36" t="s">
         <v>1657</v>
       </c>
-      <c r="B49" s="36" t="s">
+      <c r="B49" s="37" t="s">
         <v>1658</v>
       </c>
-      <c r="C49" s="35"/>
+      <c r="C49" s="36"/>
     </row>
     <row r="50" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="35" t="s">
+      <c r="A50" s="36" t="s">
         <v>1659</v>
       </c>
-      <c r="B50" s="36" t="s">
+      <c r="B50" s="37" t="s">
         <v>1660</v>
       </c>
-      <c r="C50" s="35"/>
+      <c r="C50" s="36"/>
     </row>
     <row r="51" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="35" t="s">
+      <c r="A51" s="36" t="s">
         <v>1661</v>
       </c>
-      <c r="B51" s="36" t="s">
+      <c r="B51" s="37" t="s">
         <v>1662</v>
       </c>
-      <c r="C51" s="35"/>
+      <c r="C51" s="36"/>
     </row>
     <row r="52" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="35" t="s">
+      <c r="A52" s="36" t="s">
         <v>1663</v>
       </c>
-      <c r="B52" s="36" t="s">
+      <c r="B52" s="37" t="s">
         <v>1664</v>
       </c>
-      <c r="C52" s="35"/>
+      <c r="C52" s="36"/>
     </row>
     <row r="53" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A53" s="35" t="s">
+      <c r="A53" s="36" t="s">
         <v>1665</v>
       </c>
-      <c r="B53" s="36" t="s">
+      <c r="B53" s="37" t="s">
         <v>1666</v>
       </c>
-      <c r="C53" s="35"/>
+      <c r="C53" s="36"/>
     </row>
     <row r="54" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A54" s="35" t="s">
+      <c r="A54" s="36" t="s">
         <v>1667</v>
       </c>
-      <c r="B54" s="36" t="s">
+      <c r="B54" s="37" t="s">
         <v>1668</v>
       </c>
-      <c r="C54" s="35"/>
+      <c r="C54" s="36"/>
     </row>
     <row r="55" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="35" t="s">
+      <c r="A55" s="36" t="s">
         <v>1669</v>
       </c>
-      <c r="B55" s="36" t="s">
+      <c r="B55" s="37" t="s">
         <v>1670</v>
       </c>
-      <c r="C55" s="35"/>
+      <c r="C55" s="36"/>
     </row>
     <row r="56" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="35" t="s">
+      <c r="A56" s="36" t="s">
         <v>1671</v>
       </c>
-      <c r="B56" s="36" t="s">
+      <c r="B56" s="37" t="s">
         <v>1672</v>
       </c>
-      <c r="C56" s="35"/>
+      <c r="C56" s="36"/>
     </row>
     <row r="57" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A57" s="35" t="s">
+      <c r="A57" s="36" t="s">
         <v>1673</v>
       </c>
-      <c r="B57" s="36" t="s">
+      <c r="B57" s="37" t="s">
         <v>1674</v>
       </c>
-      <c r="C57" s="35"/>
+      <c r="C57" s="36"/>
     </row>
     <row r="58" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="35" t="s">
+      <c r="A58" s="36" t="s">
         <v>1675</v>
       </c>
-      <c r="B58" s="36" t="s">
+      <c r="B58" s="37" t="s">
         <v>1676</v>
       </c>
-      <c r="C58" s="35"/>
+      <c r="C58" s="36"/>
     </row>
     <row r="59" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="35" t="s">
+      <c r="A59" s="36" t="s">
         <v>1677</v>
       </c>
-      <c r="B59" s="36" t="s">
+      <c r="B59" s="37" t="s">
         <v>1678</v>
       </c>
-      <c r="C59" s="35"/>
+      <c r="C59" s="36"/>
     </row>
     <row r="60" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="35" t="s">
+      <c r="A60" s="36" t="s">
         <v>1679</v>
       </c>
-      <c r="B60" s="36" t="s">
+      <c r="B60" s="37" t="s">
         <v>1680</v>
       </c>
-      <c r="C60" s="35"/>
+      <c r="C60" s="36"/>
     </row>
     <row r="61" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A61" s="35" t="s">
+      <c r="A61" s="36" t="s">
         <v>1681</v>
       </c>
-      <c r="B61" s="36" t="s">
+      <c r="B61" s="37" t="s">
         <v>1682</v>
       </c>
-      <c r="C61" s="35"/>
+      <c r="C61" s="36"/>
     </row>
     <row r="62" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A62" s="35" t="s">
+      <c r="A62" s="36" t="s">
         <v>1683</v>
       </c>
-      <c r="B62" s="36" t="s">
+      <c r="B62" s="37" t="s">
         <v>1684</v>
       </c>
-      <c r="C62" s="35"/>
+      <c r="C62" s="36"/>
     </row>
     <row r="63" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A63" s="35" t="s">
+      <c r="A63" s="36" t="s">
         <v>1685</v>
       </c>
-      <c r="B63" s="36" t="s">
+      <c r="B63" s="37" t="s">
         <v>1686</v>
       </c>
-      <c r="C63" s="35"/>
+      <c r="C63" s="36"/>
     </row>
     <row r="64" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A64" s="35" t="s">
+      <c r="A64" s="36" t="s">
         <v>1687</v>
       </c>
-      <c r="B64" s="36" t="s">
+      <c r="B64" s="37" t="s">
         <v>1688</v>
       </c>
-      <c r="C64" s="35"/>
+      <c r="C64" s="36"/>
     </row>
     <row r="65" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A65" s="35" t="s">
+      <c r="A65" s="36" t="s">
         <v>1689</v>
       </c>
-      <c r="B65" s="36" t="s">
+      <c r="B65" s="37" t="s">
         <v>1690</v>
       </c>
-      <c r="C65" s="35"/>
+      <c r="C65" s="36"/>
     </row>
     <row r="66" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A66" s="35" t="s">
+      <c r="A66" s="36" t="s">
         <v>1691</v>
       </c>
-      <c r="B66" s="36" t="s">
+      <c r="B66" s="37" t="s">
         <v>1692</v>
       </c>
-      <c r="C66" s="35"/>
+      <c r="C66" s="36"/>
     </row>
     <row r="67" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A67" s="35" t="s">
+      <c r="A67" s="36" t="s">
         <v>1693</v>
       </c>
-      <c r="B67" s="36" t="s">
+      <c r="B67" s="37" t="s">
         <v>1694</v>
       </c>
-      <c r="C67" s="35"/>
+      <c r="C67" s="36"/>
     </row>
     <row r="68" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A68" s="35" t="s">
+      <c r="A68" s="36" t="s">
         <v>1695</v>
       </c>
-      <c r="B68" s="36" t="s">
+      <c r="B68" s="37" t="s">
         <v>1696</v>
       </c>
-      <c r="C68" s="35"/>
+      <c r="C68" s="36"/>
     </row>
     <row r="69" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A69" s="35" t="s">
+      <c r="A69" s="36" t="s">
         <v>1697</v>
       </c>
-      <c r="B69" s="36" t="s">
+      <c r="B69" s="37" t="s">
         <v>1698</v>
       </c>
-      <c r="C69" s="35"/>
+      <c r="C69" s="36"/>
     </row>
     <row r="70" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A70" s="35" t="s">
+      <c r="A70" s="36" t="s">
         <v>1699</v>
       </c>
-      <c r="B70" s="36" t="s">
+      <c r="B70" s="37" t="s">
         <v>1700</v>
       </c>
-      <c r="C70" s="35"/>
+      <c r="C70" s="36"/>
     </row>
     <row r="71" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A71" s="35" t="s">
+      <c r="A71" s="36" t="s">
         <v>1701</v>
       </c>
-      <c r="B71" s="36" t="s">
+      <c r="B71" s="37" t="s">
         <v>1702</v>
       </c>
-      <c r="C71" s="35"/>
+      <c r="C71" s="36"/>
     </row>
     <row r="72" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A72" s="35" t="s">
+      <c r="A72" s="36" t="s">
         <v>1703</v>
       </c>
-      <c r="B72" s="36" t="s">
+      <c r="B72" s="37" t="s">
         <v>1704</v>
       </c>
-      <c r="C72" s="35"/>
+      <c r="C72" s="36"/>
     </row>
     <row r="73" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A73" s="35" t="s">
+      <c r="A73" s="36" t="s">
         <v>1705</v>
       </c>
-      <c r="B73" s="36" t="s">
+      <c r="B73" s="37" t="s">
         <v>1706</v>
       </c>
-      <c r="C73" s="35"/>
+      <c r="C73" s="36"/>
     </row>
     <row r="74" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A74" s="35" t="s">
+      <c r="A74" s="36" t="s">
         <v>1707</v>
       </c>
-      <c r="B74" s="36" t="s">
+      <c r="B74" s="37" t="s">
         <v>1708</v>
       </c>
-      <c r="C74" s="35"/>
+      <c r="C74" s="36"/>
     </row>
     <row r="75" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A75" s="35" t="s">
+      <c r="A75" s="36" t="s">
         <v>1709</v>
       </c>
-      <c r="B75" s="36" t="s">
+      <c r="B75" s="37" t="s">
         <v>1710</v>
       </c>
-      <c r="C75" s="35"/>
+      <c r="C75" s="36"/>
     </row>
     <row r="76" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A76" s="35" t="s">
+      <c r="A76" s="36" t="s">
         <v>1711</v>
       </c>
-      <c r="B76" s="36" t="s">
+      <c r="B76" s="37" t="s">
         <v>1712</v>
       </c>
-      <c r="C76" s="35"/>
+      <c r="C76" s="36"/>
     </row>
     <row r="77" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A77" s="35" t="s">
+      <c r="A77" s="36" t="s">
         <v>1713</v>
       </c>
-      <c r="B77" s="36" t="s">
+      <c r="B77" s="37" t="s">
         <v>1714</v>
       </c>
-      <c r="C77" s="35"/>
+      <c r="C77" s="36"/>
     </row>
     <row r="78" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A78" s="35" t="s">
+      <c r="A78" s="36" t="s">
         <v>1715</v>
       </c>
-      <c r="B78" s="36" t="s">
+      <c r="B78" s="37" t="s">
         <v>1716</v>
       </c>
-      <c r="C78" s="35"/>
+      <c r="C78" s="36"/>
     </row>
     <row r="79" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A79" s="35" t="s">
+      <c r="A79" s="36" t="s">
         <v>1717</v>
       </c>
-      <c r="B79" s="36" t="s">
+      <c r="B79" s="37" t="s">
         <v>1718</v>
       </c>
-      <c r="C79" s="35"/>
+      <c r="C79" s="36"/>
     </row>
     <row r="80" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A80" s="35" t="s">
+      <c r="A80" s="36" t="s">
         <v>1719</v>
       </c>
-      <c r="B80" s="36" t="s">
+      <c r="B80" s="37" t="s">
         <v>1720</v>
       </c>
-      <c r="C80" s="35"/>
+      <c r="C80" s="36"/>
     </row>
     <row r="81" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A81" s="35" t="s">
+      <c r="A81" s="36" t="s">
         <v>1721</v>
       </c>
-      <c r="B81" s="36" t="s">
+      <c r="B81" s="37" t="s">
         <v>1722</v>
       </c>
-      <c r="C81" s="35"/>
+      <c r="C81" s="36"/>
     </row>
     <row r="82" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A82" s="35" t="s">
+      <c r="A82" s="36" t="s">
         <v>1723</v>
       </c>
-      <c r="B82" s="36" t="s">
+      <c r="B82" s="37" t="s">
         <v>1724</v>
       </c>
-      <c r="C82" s="35"/>
+      <c r="C82" s="36"/>
     </row>
     <row r="83" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A83" s="35" t="s">
+      <c r="A83" s="36" t="s">
         <v>1725</v>
       </c>
-      <c r="B83" s="36" t="s">
+      <c r="B83" s="37" t="s">
         <v>1726</v>
       </c>
-      <c r="C83" s="35"/>
+      <c r="C83" s="36"/>
     </row>
     <row r="84" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A84" s="35" t="s">
+      <c r="A84" s="36" t="s">
         <v>1727</v>
       </c>
-      <c r="B84" s="36" t="s">
+      <c r="B84" s="37" t="s">
         <v>1728</v>
       </c>
-      <c r="C84" s="35"/>
+      <c r="C84" s="36"/>
     </row>
     <row r="85" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A85" s="35" t="s">
+      <c r="A85" s="36" t="s">
         <v>1729</v>
       </c>
-      <c r="B85" s="36" t="s">
+      <c r="B85" s="37" t="s">
         <v>1730</v>
       </c>
-      <c r="C85" s="35"/>
+      <c r="C85" s="36"/>
     </row>
     <row r="86" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A86" s="35" t="s">
+      <c r="A86" s="36" t="s">
         <v>1731</v>
       </c>
-      <c r="B86" s="36" t="s">
+      <c r="B86" s="37" t="s">
         <v>1732</v>
       </c>
-      <c r="C86" s="35"/>
+      <c r="C86" s="36"/>
     </row>
     <row r="87" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A87" s="35" t="s">
+      <c r="A87" s="36" t="s">
         <v>1733</v>
       </c>
-      <c r="B87" s="36" t="s">
+      <c r="B87" s="37" t="s">
         <v>1734</v>
       </c>
-      <c r="C87" s="35"/>
+      <c r="C87" s="36"/>
     </row>
     <row r="88" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A88" s="35" t="s">
+      <c r="A88" s="36" t="s">
         <v>1735</v>
       </c>
-      <c r="B88" s="36" t="s">
+      <c r="B88" s="37" t="s">
         <v>1736</v>
       </c>
-      <c r="C88" s="35"/>
+      <c r="C88" s="36"/>
     </row>
     <row r="89" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A89" s="35" t="s">
+      <c r="A89" s="36" t="s">
         <v>1737</v>
       </c>
-      <c r="B89" s="36" t="s">
+      <c r="B89" s="37" t="s">
         <v>1738</v>
       </c>
-      <c r="C89" s="35"/>
+      <c r="C89" s="36"/>
     </row>
     <row r="90" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A90" s="35" t="s">
+      <c r="A90" s="36" t="s">
         <v>1739</v>
       </c>
-      <c r="B90" s="36" t="s">
+      <c r="B90" s="37" t="s">
         <v>1740</v>
       </c>
-      <c r="C90" s="35"/>
+      <c r="C90" s="36"/>
     </row>
     <row r="91" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A91" s="35" t="s">
+      <c r="A91" s="36" t="s">
         <v>1741</v>
       </c>
-      <c r="B91" s="36" t="s">
+      <c r="B91" s="37" t="s">
         <v>1742</v>
       </c>
-      <c r="C91" s="35"/>
+      <c r="C91" s="36"/>
     </row>
     <row r="92" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A92" s="35" t="s">
+      <c r="A92" s="36" t="s">
         <v>1743</v>
       </c>
-      <c r="B92" s="36" t="s">
+      <c r="B92" s="37" t="s">
         <v>1744</v>
       </c>
-      <c r="C92" s="35"/>
+      <c r="C92" s="36"/>
     </row>
     <row r="93" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A93" s="35" t="s">
+      <c r="A93" s="36" t="s">
         <v>1745</v>
       </c>
-      <c r="B93" s="36" t="s">
+      <c r="B93" s="37" t="s">
         <v>1746</v>
       </c>
-      <c r="C93" s="35"/>
+      <c r="C93" s="36"/>
     </row>
     <row r="94" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A94" s="35" t="s">
+      <c r="A94" s="36" t="s">
         <v>1747</v>
       </c>
-      <c r="B94" s="36" t="s">
+      <c r="B94" s="37" t="s">
         <v>1748</v>
       </c>
-      <c r="C94" s="35"/>
+      <c r="C94" s="36"/>
     </row>
     <row r="95" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A95" s="35" t="s">
+      <c r="A95" s="36" t="s">
         <v>1749</v>
       </c>
-      <c r="B95" s="36" t="s">
+      <c r="B95" s="37" t="s">
         <v>1750</v>
       </c>
-      <c r="C95" s="35"/>
+      <c r="C95" s="36"/>
     </row>
     <row r="96" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A96" s="35" t="s">
+      <c r="A96" s="36" t="s">
         <v>1751</v>
       </c>
-      <c r="B96" s="36" t="s">
+      <c r="B96" s="37" t="s">
         <v>1752</v>
       </c>
-      <c r="C96" s="35"/>
+      <c r="C96" s="36"/>
     </row>
     <row r="97" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A97" s="35" t="s">
+      <c r="A97" s="36" t="s">
         <v>1753</v>
       </c>
-      <c r="B97" s="36" t="s">
+      <c r="B97" s="37" t="s">
         <v>1754</v>
       </c>
-      <c r="C97" s="35"/>
+      <c r="C97" s="36"/>
     </row>
     <row r="98" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A98" s="35" t="s">
+      <c r="A98" s="36" t="s">
         <v>1755</v>
       </c>
-      <c r="B98" s="36" t="s">
+      <c r="B98" s="37" t="s">
         <v>1756</v>
       </c>
-      <c r="C98" s="35"/>
+      <c r="C98" s="36"/>
     </row>
     <row r="99" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A99" s="35" t="s">
+      <c r="A99" s="36" t="s">
         <v>1757</v>
       </c>
-      <c r="B99" s="36" t="s">
+      <c r="B99" s="37" t="s">
         <v>1758</v>
       </c>
-      <c r="C99" s="35"/>
+      <c r="C99" s="36"/>
     </row>
     <row r="100" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A100" s="35" t="s">
+      <c r="A100" s="36" t="s">
         <v>1759</v>
       </c>
-      <c r="B100" s="36" t="s">
+      <c r="B100" s="37" t="s">
         <v>1760</v>
       </c>
-      <c r="C100" s="35"/>
+      <c r="C100" s="36"/>
     </row>
     <row r="101" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A101" s="35" t="s">
+      <c r="A101" s="36" t="s">
         <v>1761</v>
       </c>
-      <c r="B101" s="36" t="s">
+      <c r="B101" s="37" t="s">
         <v>1762</v>
       </c>
-      <c r="C101" s="35"/>
+      <c r="C101" s="36"/>
     </row>
     <row r="102" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A102" s="35" t="s">
+      <c r="A102" s="36" t="s">
         <v>1763</v>
       </c>
-      <c r="B102" s="36" t="s">
+      <c r="B102" s="37" t="s">
         <v>1764</v>
       </c>
-      <c r="C102" s="35"/>
+      <c r="C102" s="36"/>
     </row>
     <row r="103" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A103" s="35" t="s">
+      <c r="A103" s="36" t="s">
         <v>1765</v>
       </c>
-      <c r="B103" s="36" t="s">
+      <c r="B103" s="37" t="s">
         <v>1766</v>
       </c>
-      <c r="C103" s="35"/>
+      <c r="C103" s="36"/>
     </row>
     <row r="104" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A104" s="35" t="s">
+      <c r="A104" s="36" t="s">
         <v>1767</v>
       </c>
-      <c r="B104" s="36" t="s">
+      <c r="B104" s="37" t="s">
         <v>1768</v>
       </c>
-      <c r="C104" s="35"/>
+      <c r="C104" s="36"/>
     </row>
     <row r="105" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A105" s="35" t="s">
+      <c r="A105" s="36" t="s">
         <v>1769</v>
       </c>
-      <c r="B105" s="36" t="s">
+      <c r="B105" s="37" t="s">
         <v>54</v>
       </c>
-      <c r="C105" s="36" t="s">
+      <c r="C105" s="37" t="s">
         <v>1770</v>
       </c>
     </row>
@@ -35288,14 +35291,14 @@
       <c r="F89" s="6"/>
     </row>
     <row r="90" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A90" s="6" t="s">
+      <c r="A90" s="33" t="s">
         <v>851</v>
       </c>
-      <c r="B90" s="6"/>
-      <c r="C90" s="6"/>
-      <c r="D90" s="6"/>
-      <c r="E90" s="6"/>
-      <c r="F90" s="6"/>
+      <c r="B90" s="33"/>
+      <c r="C90" s="33"/>
+      <c r="D90" s="33"/>
+      <c r="E90" s="33"/>
+      <c r="F90" s="33"/>
     </row>
     <row r="91" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="4" t="s">
@@ -35410,14 +35413,14 @@
       <c r="F97" s="22"/>
     </row>
     <row r="98" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A98" s="6" t="s">
+      <c r="A98" s="33" t="s">
         <v>864</v>
       </c>
-      <c r="B98" s="6"/>
-      <c r="C98" s="6"/>
-      <c r="D98" s="6"/>
-      <c r="E98" s="6"/>
-      <c r="F98" s="6"/>
+      <c r="B98" s="33"/>
+      <c r="C98" s="33"/>
+      <c r="D98" s="33"/>
+      <c r="E98" s="33"/>
+      <c r="F98" s="33"/>
     </row>
     <row r="99" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A99" s="4" t="s">
@@ -36178,7 +36181,7 @@
       <c r="D153" s="16" t="s">
         <v>564</v>
       </c>
-      <c r="E153" s="33" t="s">
+      <c r="E153" s="34" t="s">
         <v>958</v>
       </c>
       <c r="F153" s="18" t="s">
@@ -36194,7 +36197,7 @@
       <c r="D154" s="16" t="s">
         <v>564</v>
       </c>
-      <c r="E154" s="33" t="s">
+      <c r="E154" s="34" t="s">
         <v>961</v>
       </c>
       <c r="F154" s="18" t="s">
@@ -41329,321 +41332,321 @@
   <sheetFormatPr defaultColWidth="8.62109375" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="35" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="34" t="s">
+      <c r="B1" s="35" t="s">
         <v>412</v>
       </c>
-      <c r="C1" s="34" t="s">
+      <c r="C1" s="35" t="s">
         <v>1497</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="35" t="s">
+      <c r="A2" s="36" t="s">
         <v>1498</v>
       </c>
-      <c r="B2" s="36" t="s">
+      <c r="B2" s="37" t="s">
         <v>1499</v>
       </c>
-      <c r="C2" s="35" t="s">
+      <c r="C2" s="36" t="s">
         <v>1500</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="35" t="s">
+      <c r="A3" s="36" t="s">
         <v>76</v>
       </c>
-      <c r="B3" s="36" t="s">
+      <c r="B3" s="37" t="s">
         <v>1501</v>
       </c>
-      <c r="C3" s="35" t="s">
+      <c r="C3" s="36" t="s">
         <v>1502</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="35" t="s">
+      <c r="A4" s="36" t="s">
         <v>84</v>
       </c>
-      <c r="B4" s="36" t="s">
+      <c r="B4" s="37" t="s">
         <v>1503</v>
       </c>
-      <c r="C4" s="35" t="s">
+      <c r="C4" s="36" t="s">
         <v>1504</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="35" t="s">
+      <c r="A5" s="36" t="s">
         <v>90</v>
       </c>
-      <c r="B5" s="36" t="s">
+      <c r="B5" s="37" t="s">
         <v>1505</v>
       </c>
-      <c r="C5" s="35" t="s">
+      <c r="C5" s="36" t="s">
         <v>1506</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="35" t="s">
+      <c r="A6" s="36" t="s">
         <v>101</v>
       </c>
-      <c r="B6" s="36" t="s">
+      <c r="B6" s="37" t="s">
         <v>1507</v>
       </c>
-      <c r="C6" s="35" t="s">
+      <c r="C6" s="36" t="s">
         <v>1508</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="35" t="s">
+      <c r="A7" s="36" t="s">
         <v>110</v>
       </c>
-      <c r="B7" s="36" t="s">
+      <c r="B7" s="37" t="s">
         <v>1509</v>
       </c>
-      <c r="C7" s="35" t="s">
+      <c r="C7" s="36" t="s">
         <v>1510</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="35" t="s">
+      <c r="A8" s="36" t="s">
         <v>473</v>
       </c>
-      <c r="B8" s="36" t="s">
+      <c r="B8" s="37" t="s">
         <v>1511</v>
       </c>
-      <c r="C8" s="35" t="s">
+      <c r="C8" s="36" t="s">
         <v>1512</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="35" t="s">
+      <c r="A9" s="36" t="s">
         <v>476</v>
       </c>
-      <c r="B9" s="36" t="s">
+      <c r="B9" s="37" t="s">
         <v>1513</v>
       </c>
-      <c r="C9" s="35" t="s">
+      <c r="C9" s="36" t="s">
         <v>1514</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="35" t="s">
+      <c r="A10" s="36" t="s">
         <v>746</v>
       </c>
-      <c r="B10" s="36" t="s">
+      <c r="B10" s="37" t="s">
         <v>1515</v>
       </c>
-      <c r="C10" s="35" t="s">
+      <c r="C10" s="36" t="s">
         <v>1516</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="35" t="s">
+      <c r="A11" s="36" t="s">
         <v>750</v>
       </c>
-      <c r="B11" s="36" t="s">
+      <c r="B11" s="37" t="s">
         <v>1517</v>
       </c>
-      <c r="C11" s="35" t="s">
+      <c r="C11" s="36" t="s">
         <v>1518</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="35" t="s">
+      <c r="A12" s="36" t="s">
         <v>753</v>
       </c>
-      <c r="B12" s="36" t="s">
+      <c r="B12" s="37" t="s">
         <v>1519</v>
       </c>
-      <c r="C12" s="35" t="s">
+      <c r="C12" s="36" t="s">
         <v>1520</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="35" t="s">
+      <c r="A13" s="36" t="s">
         <v>756</v>
       </c>
-      <c r="B13" s="36" t="s">
+      <c r="B13" s="37" t="s">
         <v>1521</v>
       </c>
-      <c r="C13" s="35" t="s">
+      <c r="C13" s="36" t="s">
         <v>1522</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="35" t="s">
+      <c r="A14" s="36" t="s">
         <v>760</v>
       </c>
-      <c r="B14" s="36" t="s">
+      <c r="B14" s="37" t="s">
         <v>1523</v>
       </c>
-      <c r="C14" s="35" t="s">
+      <c r="C14" s="36" t="s">
         <v>1524</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="35" t="s">
+      <c r="A15" s="36" t="s">
         <v>764</v>
       </c>
-      <c r="B15" s="36" t="s">
+      <c r="B15" s="37" t="s">
         <v>1525</v>
       </c>
-      <c r="C15" s="35" t="s">
+      <c r="C15" s="36" t="s">
         <v>1526</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="35" t="s">
+      <c r="A16" s="36" t="s">
         <v>1527</v>
       </c>
-      <c r="B16" s="36" t="s">
+      <c r="B16" s="37" t="s">
         <v>1528</v>
       </c>
-      <c r="C16" s="35" t="s">
+      <c r="C16" s="36" t="s">
         <v>1529</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="35" t="s">
+      <c r="A17" s="36" t="s">
         <v>1530</v>
       </c>
-      <c r="B17" s="36" t="s">
+      <c r="B17" s="37" t="s">
         <v>1531</v>
       </c>
-      <c r="C17" s="35" t="s">
+      <c r="C17" s="36" t="s">
         <v>1532</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="35" t="s">
+      <c r="A18" s="36" t="s">
         <v>119</v>
       </c>
-      <c r="B18" s="36" t="s">
+      <c r="B18" s="37" t="s">
         <v>1533</v>
       </c>
-      <c r="C18" s="35" t="s">
+      <c r="C18" s="36" t="s">
         <v>1534</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="35" t="s">
+      <c r="A19" s="36" t="s">
         <v>125</v>
       </c>
-      <c r="B19" s="36" t="s">
+      <c r="B19" s="37" t="s">
         <v>1535</v>
       </c>
-      <c r="C19" s="35" t="s">
+      <c r="C19" s="36" t="s">
         <v>1536</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="35" t="s">
+      <c r="A20" s="36" t="s">
         <v>134</v>
       </c>
-      <c r="B20" s="36" t="s">
+      <c r="B20" s="37" t="s">
         <v>1537</v>
       </c>
-      <c r="C20" s="35" t="s">
+      <c r="C20" s="36" t="s">
         <v>1538</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="35" t="s">
+      <c r="A21" s="36" t="s">
         <v>143</v>
       </c>
-      <c r="B21" s="36" t="s">
+      <c r="B21" s="37" t="s">
         <v>1539</v>
       </c>
-      <c r="C21" s="35" t="s">
+      <c r="C21" s="36" t="s">
         <v>1540</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="35" t="s">
+      <c r="A22" s="36" t="s">
         <v>1086</v>
       </c>
-      <c r="B22" s="36" t="s">
+      <c r="B22" s="37" t="s">
         <v>1541</v>
       </c>
-      <c r="C22" s="35" t="s">
+      <c r="C22" s="36" t="s">
         <v>1542</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="35" t="s">
+      <c r="A23" s="36" t="s">
         <v>1090</v>
       </c>
-      <c r="B23" s="36" t="s">
+      <c r="B23" s="37" t="s">
         <v>1543</v>
       </c>
-      <c r="C23" s="35" t="s">
+      <c r="C23" s="36" t="s">
         <v>1544</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="35" t="s">
+      <c r="A24" s="36" t="s">
         <v>1093</v>
       </c>
-      <c r="B24" s="36" t="s">
+      <c r="B24" s="37" t="s">
         <v>1545</v>
       </c>
-      <c r="C24" s="35" t="s">
+      <c r="C24" s="36" t="s">
         <v>1546</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="35" t="s">
+      <c r="A25" s="36" t="s">
         <v>1547</v>
       </c>
-      <c r="B25" s="36" t="s">
+      <c r="B25" s="37" t="s">
         <v>1548</v>
       </c>
-      <c r="C25" s="35" t="s">
+      <c r="C25" s="36" t="s">
         <v>1549</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="35" t="s">
+      <c r="A26" s="36" t="s">
         <v>1550</v>
       </c>
-      <c r="B26" s="36" t="s">
+      <c r="B26" s="37" t="s">
         <v>1551</v>
       </c>
-      <c r="C26" s="35" t="s">
+      <c r="C26" s="36" t="s">
         <v>1552</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="35" t="s">
+      <c r="A27" s="36" t="s">
         <v>1553</v>
       </c>
-      <c r="B27" s="36" t="s">
+      <c r="B27" s="37" t="s">
         <v>1554</v>
       </c>
-      <c r="C27" s="35" t="s">
+      <c r="C27" s="36" t="s">
         <v>1555</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="35" t="s">
+      <c r="A28" s="36" t="s">
         <v>1556</v>
       </c>
-      <c r="B28" s="36" t="s">
+      <c r="B28" s="37" t="s">
         <v>1557</v>
       </c>
-      <c r="C28" s="35" t="s">
+      <c r="C28" s="36" t="s">
         <v>1558</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="35" t="s">
+      <c r="A29" s="36" t="s">
         <v>1559</v>
       </c>
-      <c r="B29" s="36" t="s">
+      <c r="B29" s="37" t="s">
         <v>54</v>
       </c>
-      <c r="C29" s="36" t="s">
+      <c r="C29" s="37" t="s">
         <v>1560</v>
       </c>
     </row>

</xml_diff>